<commit_message>
Atualização automática do LAIA - Samuel Camargos - Revisão da avaliação dos fatores dos impactos
</commit_message>
<xml_diff>
--- a/dados/LAIA.xlsx
+++ b/dados/LAIA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samuel.camargo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA3049E-43B8-4CAE-8CB1-D6B514F10CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF97FFBB-4898-49B8-A80C-735EA81B3CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2958,6 +2958,42 @@
     <xf numFmtId="0" fontId="48" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2975,9 +3011,6 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3023,39 +3056,6 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="9" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -3353,7 +3353,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[PIU - LAIA.xlsx]Significância-processo-aspecto!Tabela dinâmica3</c:name>
+    <c:name>[LAIA.xlsx]Significância-processo-aspecto!Tabela dinâmica3</c:name>
     <c:fmtId val="0"/>
   </c:pivotSource>
   <c:chart>
@@ -24812,7 +24812,7 @@
         <v>270</v>
       </c>
       <c r="S36" s="75" t="str">
-        <f t="shared" ref="S36:S67" si="5">IF(R36&gt;400,"Insustentável (risco extremo)", IF(R36&gt;200,"Significativo (risco muito alto)", IF(R36&gt;70,"Significativo (alto risco)", IF(R36&gt;21,"Significativo (risco médio)", "Insignificante"))))</f>
+        <f t="shared" ref="S36:S59" si="5">IF(R36&gt;400,"Insustentável (risco extremo)", IF(R36&gt;200,"Significativo (risco muito alto)", IF(R36&gt;70,"Significativo (alto risco)", IF(R36&gt;21,"Significativo (risco médio)", "Insignificante"))))</f>
         <v>Significativo (risco muito alto)</v>
       </c>
       <c r="T36" s="67" t="s">
@@ -24838,7 +24838,7 @@
         <v>54</v>
       </c>
       <c r="AA36" s="75" t="str">
-        <f t="shared" ref="AA36:AA67" si="6">IF(Z36&gt;400,"Insustentável (risco extremo)", IF(Z36&gt;200,"Significativo (risco muito alto)", IF(Z36&gt;70,"Significativo (alto risco)", IF(Z36&gt;21,"Significativo (risco médio)", "Insignificante"))))</f>
+        <f t="shared" ref="AA36:AA59" si="6">IF(Z36&gt;400,"Insustentável (risco extremo)", IF(Z36&gt;200,"Significativo (risco muito alto)", IF(Z36&gt;70,"Significativo (alto risco)", IF(Z36&gt;21,"Significativo (risco médio)", "Insignificante"))))</f>
         <v>Significativo (risco médio)</v>
       </c>
       <c r="AB36" s="67" t="s">
@@ -25882,18 +25882,18 @@
         <v>3</v>
       </c>
       <c r="P48" s="72">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Q48" s="73">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R48" s="74">
         <f t="shared" si="3"/>
-        <v>126</v>
+        <v>27</v>
       </c>
       <c r="S48" s="75" t="str">
         <f t="shared" si="5"/>
-        <v>Significativo (alto risco)</v>
+        <v>Significativo (risco médio)</v>
       </c>
       <c r="T48" s="67" t="s">
         <v>296</v>
@@ -25905,17 +25905,17 @@
         <v>298</v>
       </c>
       <c r="W48" s="76">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X48" s="72">
         <v>3</v>
       </c>
       <c r="Y48" s="73">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="Z48" s="77">
         <f t="shared" si="4"/>
-        <v>0.30000000000000004</v>
+        <v>9</v>
       </c>
       <c r="AA48" s="75" t="str">
         <f t="shared" si="6"/>
@@ -26150,14 +26150,14 @@
         <v>2</v>
       </c>
       <c r="P51" s="72">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Q51" s="73">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="R51" s="74">
         <f t="shared" si="3"/>
-        <v>1.4000000000000001</v>
+        <v>6</v>
       </c>
       <c r="S51" s="75" t="str">
         <f t="shared" si="5"/>
@@ -26179,11 +26179,11 @@
         <v>3</v>
       </c>
       <c r="Y51" s="73">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Z51" s="77">
         <f t="shared" si="4"/>
-        <v>0.60000000000000009</v>
+        <v>3</v>
       </c>
       <c r="AA51" s="75" t="str">
         <f t="shared" si="6"/>
@@ -26283,7 +26283,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="53" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="53" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A53" s="50">
         <v>67</v>
       </c>
@@ -26327,17 +26327,17 @@
         <v>33</v>
       </c>
       <c r="O53" s="71">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P53" s="72">
         <v>3</v>
       </c>
       <c r="Q53" s="73">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="R53" s="74">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="S53" s="75" t="str">
         <f t="shared" si="5"/>
@@ -26359,11 +26359,11 @@
         <v>3</v>
       </c>
       <c r="Y53" s="73">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Z53" s="77">
         <f t="shared" si="4"/>
-        <v>0.60000000000000009</v>
+        <v>3</v>
       </c>
       <c r="AA53" s="75" t="str">
         <f t="shared" si="6"/>
@@ -26373,7 +26373,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="54" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" customHeight="1" x14ac:dyDescent="1.45">
+    <row r="54" spans="1:28" s="54" customFormat="1" ht="382.5" customHeight="1" x14ac:dyDescent="1.45">
       <c r="A54" s="50">
         <v>69</v>
       </c>
@@ -26417,17 +26417,17 @@
         <v>43</v>
       </c>
       <c r="O54" s="71">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P54" s="72">
         <v>3</v>
       </c>
       <c r="Q54" s="73">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="R54" s="74">
         <f t="shared" si="3"/>
-        <v>1.2000000000000002</v>
+        <v>9</v>
       </c>
       <c r="S54" s="75" t="str">
         <f t="shared" si="5"/>
@@ -26449,11 +26449,11 @@
         <v>3</v>
       </c>
       <c r="Y54" s="73">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Z54" s="77">
         <f t="shared" si="4"/>
-        <v>0.60000000000000009</v>
+        <v>3</v>
       </c>
       <c r="AA54" s="75" t="str">
         <f t="shared" si="6"/>
@@ -26463,7 +26463,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="55" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="55" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A55" s="50">
         <v>70</v>
       </c>
@@ -26507,7 +26507,7 @@
         <v>35</v>
       </c>
       <c r="O55" s="71">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="P55" s="72">
         <v>3</v>
@@ -26517,7 +26517,7 @@
       </c>
       <c r="R55" s="74">
         <f t="shared" si="3"/>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="S55" s="75" t="str">
         <f t="shared" si="5"/>
@@ -26553,7 +26553,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="56" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="56" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A56" s="50">
         <v>72</v>
       </c>
@@ -26643,7 +26643,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="57" spans="1:28" s="54" customFormat="1" ht="409.5" hidden="1" customHeight="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="57" spans="1:28" s="54" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A57" s="50">
         <v>73</v>
       </c>
@@ -26690,14 +26690,14 @@
         <v>10</v>
       </c>
       <c r="P57" s="72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q57" s="73">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="R57" s="74">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="S57" s="75" t="str">
         <f t="shared" si="5"/>
@@ -26733,7 +26733,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="58" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A58" s="50">
         <v>74</v>
       </c>
@@ -26823,7 +26823,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="59" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="59" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A59" s="50">
         <v>75</v>
       </c>
@@ -26913,7 +26913,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="60" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="60" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A60" s="50">
         <v>76</v>
       </c>
@@ -26999,7 +26999,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="61" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="61" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A61" s="50">
         <v>77</v>
       </c>
@@ -27089,7 +27089,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="62" spans="1:28" s="54" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="62" spans="1:28" s="54" customFormat="1" ht="409.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A62" s="50">
         <v>78</v>
       </c>
@@ -27179,7 +27179,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="63" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
       <c r="A63" s="50">
         <v>79</v>
       </c>
@@ -29956,7 +29956,7 @@
         <v>0.2</v>
       </c>
       <c r="Z93" s="77">
-        <f t="shared" ref="Z93:Z124" si="13">PRODUCT(W93:Y93)</f>
+        <f t="shared" ref="Z93:Z119" si="13">PRODUCT(W93:Y93)</f>
         <v>1.2000000000000002</v>
       </c>
       <c r="AA93" s="75" t="str">
@@ -34102,7 +34102,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="140" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="140" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A140" s="50">
         <v>190</v>
       </c>
@@ -34192,7 +34192,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="141" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="141" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A141" s="50">
         <v>192</v>
       </c>
@@ -34282,7 +34282,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="142" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="142" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A142" s="50"/>
       <c r="B142" s="81" t="s">
         <v>26</v>
@@ -34370,7 +34370,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="143" spans="1:28" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="143" spans="1:28" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A143" s="50">
         <v>193</v>
       </c>
@@ -34460,7 +34460,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="144" spans="1:28" s="54" customFormat="1" ht="409.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="144" spans="1:28" s="54" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A144" s="50">
         <v>197</v>
       </c>
@@ -34550,7 +34550,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="145" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="145" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A145" s="53">
         <v>201</v>
       </c>
@@ -34641,7 +34641,7 @@
       </c>
       <c r="AC145" s="59"/>
     </row>
-    <row r="146" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="146" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A146" s="53">
         <v>202</v>
       </c>
@@ -34732,7 +34732,7 @@
       </c>
       <c r="AC146" s="59"/>
     </row>
-    <row r="147" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="147" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A147" s="53">
         <v>203</v>
       </c>
@@ -34823,7 +34823,7 @@
       </c>
       <c r="AC147" s="59"/>
     </row>
-    <row r="148" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="148" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A148" s="53">
         <v>205</v>
       </c>
@@ -34914,7 +34914,7 @@
       </c>
       <c r="AC148" s="59"/>
     </row>
-    <row r="149" spans="1:29" s="54" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="1.1000000000000001">
+    <row r="149" spans="1:29" s="54" customFormat="1" ht="409.6" hidden="1" customHeight="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A149" s="53"/>
       <c r="B149" s="81" t="s">
         <v>26</v>
@@ -35003,7 +35003,7 @@
       </c>
       <c r="AC149" s="59"/>
     </row>
-    <row r="150" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="150" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A150" s="53">
         <v>208</v>
       </c>
@@ -35094,7 +35094,7 @@
       </c>
       <c r="AC150" s="59"/>
     </row>
-    <row r="151" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="151" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A151" s="53">
         <v>209</v>
       </c>
@@ -35185,7 +35185,7 @@
       </c>
       <c r="AC151" s="59"/>
     </row>
-    <row r="152" spans="1:29" s="54" customFormat="1" ht="409.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="152" spans="1:29" s="54" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A152" s="53">
         <v>210</v>
       </c>
@@ -35276,7 +35276,7 @@
       </c>
       <c r="AC152" s="56"/>
     </row>
-    <row r="153" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="153" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A153" s="53">
         <v>211</v>
       </c>
@@ -35367,7 +35367,7 @@
       </c>
       <c r="AC153" s="56"/>
     </row>
-    <row r="154" spans="1:29" s="54" customFormat="1" ht="409.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="154" spans="1:29" s="54" customFormat="1" ht="409.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A154" s="53">
         <v>213</v>
       </c>
@@ -35458,7 +35458,7 @@
       </c>
       <c r="AC154" s="56"/>
     </row>
-    <row r="155" spans="1:29" s="54" customFormat="1" ht="306" x14ac:dyDescent="1.1000000000000001">
+    <row r="155" spans="1:29" s="54" customFormat="1" ht="306" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="B155" s="69" t="s">
         <v>26</v>
       </c>
@@ -35545,7 +35545,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="156" spans="1:29" s="54" customFormat="1" ht="382.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="156" spans="1:29" s="54" customFormat="1" ht="382.5" hidden="1" x14ac:dyDescent="1.1000000000000001">
       <c r="B156" s="81" t="s">
         <v>26</v>
       </c>
@@ -35640,8 +35640,7 @@
   <autoFilter ref="B3:AB156" xr:uid="{F9A4741E-2134-4562-B632-CA537B03EF9D}">
     <filterColumn colId="1">
       <filters>
-        <filter val="Torrefação"/>
-        <filter val="Torrefação, Moagem, Café Cru"/>
+        <filter val="Geral"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:AB156">
@@ -37140,47 +37139,47 @@
     <row r="1" spans="1:20" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:20" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
-      <c r="B2" s="139" t="s">
+      <c r="B2" s="117" t="s">
         <v>211</v>
       </c>
-      <c r="C2" s="139"/>
-      <c r="D2" s="140"/>
+      <c r="C2" s="117"/>
+      <c r="D2" s="118"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="141" t="s">
+      <c r="F2" s="119" t="s">
         <v>212</v>
       </c>
-      <c r="G2" s="142"/>
-      <c r="H2" s="142"/>
-      <c r="I2" s="142"/>
-      <c r="J2" s="142"/>
-      <c r="K2" s="142"/>
-      <c r="L2" s="142"/>
-      <c r="M2" s="142"/>
-      <c r="N2" s="142"/>
-      <c r="O2" s="142"/>
-      <c r="P2" s="142"/>
-      <c r="Q2" s="142"/>
-      <c r="R2" s="142"/>
-      <c r="S2" s="142"/>
-      <c r="T2" s="143"/>
+      <c r="G2" s="120"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="120"/>
+      <c r="J2" s="120"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="120"/>
+      <c r="M2" s="120"/>
+      <c r="N2" s="120"/>
+      <c r="O2" s="120"/>
+      <c r="P2" s="120"/>
+      <c r="Q2" s="120"/>
+      <c r="R2" s="120"/>
+      <c r="S2" s="120"/>
+      <c r="T2" s="121"/>
     </row>
     <row r="3" spans="1:20" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="123"/>
-      <c r="C3" s="123"/>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="123"/>
-      <c r="L3" s="123"/>
-      <c r="M3" s="123"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
-      <c r="P3" s="123"/>
-      <c r="Q3" s="123"/>
+      <c r="B3" s="122"/>
+      <c r="C3" s="122"/>
+      <c r="D3" s="122"/>
+      <c r="E3" s="122"/>
+      <c r="F3" s="122"/>
+      <c r="G3" s="122"/>
+      <c r="H3" s="122"/>
+      <c r="I3" s="122"/>
+      <c r="J3" s="122"/>
+      <c r="K3" s="122"/>
+      <c r="L3" s="122"/>
+      <c r="M3" s="122"/>
+      <c r="N3" s="122"/>
+      <c r="O3" s="122"/>
+      <c r="P3" s="122"/>
+      <c r="Q3" s="122"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
@@ -37199,10 +37198,10 @@
       <c r="H4" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="J4" s="144" t="s">
+      <c r="J4" s="123" t="s">
         <v>216</v>
       </c>
-      <c r="K4" s="145"/>
+      <c r="K4" s="124"/>
       <c r="M4" s="7">
         <f>IF(M18=6,H16,IF(M18=5,H14,IF(M18=4,H12,IF(M18=3,H10,IF(M18=2,H8,IF(M18=1,H6,""))))))</f>
         <v>10</v>
@@ -37585,27 +37584,27 @@
       <c r="T23" s="11"/>
     </row>
     <row r="24" spans="2:20" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="146" t="s">
+      <c r="B24" s="125" t="s">
         <v>243</v>
       </c>
-      <c r="C24" s="147"/>
-      <c r="D24" s="148"/>
+      <c r="C24" s="126"/>
+      <c r="D24" s="127"/>
       <c r="F24" s="26" t="e">
         <f>(F4*M4)*S4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H24" s="149" t="s">
+      <c r="H24" s="128" t="s">
         <v>244</v>
       </c>
-      <c r="I24" s="147"/>
-      <c r="J24" s="147"/>
-      <c r="K24" s="147"/>
-      <c r="L24" s="147"/>
-      <c r="M24" s="147"/>
-      <c r="N24" s="147"/>
-      <c r="O24" s="147"/>
-      <c r="P24" s="147"/>
-      <c r="Q24" s="148"/>
+      <c r="I24" s="126"/>
+      <c r="J24" s="126"/>
+      <c r="K24" s="126"/>
+      <c r="L24" s="126"/>
+      <c r="M24" s="126"/>
+      <c r="N24" s="126"/>
+      <c r="O24" s="126"/>
+      <c r="P24" s="126"/>
+      <c r="Q24" s="127"/>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
@@ -37616,27 +37615,27 @@
       <c r="D25" s="27"/>
     </row>
     <row r="26" spans="2:20" ht="34.5" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="B26" s="124" t="s">
+      <c r="B26" s="135" t="s">
         <v>245</v>
       </c>
-      <c r="C26" s="125"/>
-      <c r="D26" s="126"/>
+      <c r="C26" s="136"/>
+      <c r="D26" s="137"/>
       <c r="F26" s="28" t="e">
         <f>IF($F$24&gt;=400,"&gt;","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H26" s="127" t="s">
+      <c r="H26" s="138" t="s">
         <v>246</v>
       </c>
-      <c r="I26" s="128"/>
-      <c r="J26" s="128"/>
-      <c r="K26" s="128"/>
-      <c r="L26" s="128"/>
-      <c r="M26" s="128"/>
-      <c r="N26" s="128"/>
-      <c r="O26" s="128"/>
-      <c r="P26" s="128"/>
-      <c r="Q26" s="129"/>
+      <c r="I26" s="139"/>
+      <c r="J26" s="139"/>
+      <c r="K26" s="139"/>
+      <c r="L26" s="139"/>
+      <c r="M26" s="139"/>
+      <c r="N26" s="139"/>
+      <c r="O26" s="139"/>
+      <c r="P26" s="139"/>
+      <c r="Q26" s="140"/>
       <c r="R26" s="1"/>
       <c r="S26" s="28" t="e">
         <f>IF($F$24&gt;=400,"&lt;","")</f>
@@ -37664,23 +37663,23 @@
       <c r="T27" s="1"/>
     </row>
     <row r="28" spans="2:20" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="136" t="s">
+      <c r="B28" s="147" t="s">
         <v>247</v>
       </c>
-      <c r="C28" s="137"/>
-      <c r="D28" s="138"/>
-      <c r="H28" s="127" t="s">
+      <c r="C28" s="148"/>
+      <c r="D28" s="149"/>
+      <c r="H28" s="138" t="s">
         <v>248</v>
       </c>
-      <c r="I28" s="128"/>
-      <c r="J28" s="128"/>
-      <c r="K28" s="128"/>
-      <c r="L28" s="128"/>
-      <c r="M28" s="128"/>
-      <c r="N28" s="128"/>
-      <c r="O28" s="128"/>
-      <c r="P28" s="128"/>
-      <c r="Q28" s="129"/>
+      <c r="I28" s="139"/>
+      <c r="J28" s="139"/>
+      <c r="K28" s="139"/>
+      <c r="L28" s="139"/>
+      <c r="M28" s="139"/>
+      <c r="N28" s="139"/>
+      <c r="O28" s="139"/>
+      <c r="P28" s="139"/>
+      <c r="Q28" s="140"/>
     </row>
     <row r="29" spans="2:20" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="27"/>
@@ -37698,27 +37697,27 @@
       <c r="Q29" s="27"/>
     </row>
     <row r="30" spans="2:20" ht="33.75" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="B30" s="130" t="s">
+      <c r="B30" s="141" t="s">
         <v>249</v>
       </c>
-      <c r="C30" s="131"/>
-      <c r="D30" s="132"/>
+      <c r="C30" s="142"/>
+      <c r="D30" s="143"/>
       <c r="F30" s="28" t="e">
         <f>IF(AND($F24&lt;400,$F$24&gt;=200),"&gt;","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H30" s="120" t="s">
+      <c r="H30" s="132" t="s">
         <v>250</v>
       </c>
-      <c r="I30" s="121"/>
-      <c r="J30" s="121"/>
-      <c r="K30" s="121"/>
-      <c r="L30" s="121"/>
-      <c r="M30" s="121"/>
-      <c r="N30" s="121"/>
-      <c r="O30" s="121"/>
-      <c r="P30" s="121"/>
-      <c r="Q30" s="122"/>
+      <c r="I30" s="133"/>
+      <c r="J30" s="133"/>
+      <c r="K30" s="133"/>
+      <c r="L30" s="133"/>
+      <c r="M30" s="133"/>
+      <c r="N30" s="133"/>
+      <c r="O30" s="133"/>
+      <c r="P30" s="133"/>
+      <c r="Q30" s="134"/>
       <c r="R30" s="1"/>
       <c r="S30" s="28" t="e">
         <f>IF(AND($F24&lt;400,$F$24&gt;=200),"&lt;","")</f>
@@ -37742,27 +37741,27 @@
       <c r="Q31" s="27"/>
     </row>
     <row r="32" spans="2:20" ht="31.5" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="B32" s="133" t="s">
+      <c r="B32" s="144" t="s">
         <v>251</v>
       </c>
-      <c r="C32" s="134"/>
-      <c r="D32" s="135"/>
+      <c r="C32" s="145"/>
+      <c r="D32" s="146"/>
       <c r="F32" s="28" t="e">
         <f>IF(AND($F$24&lt;200,$F$24&gt;=70),"&gt;","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H32" s="120" t="s">
+      <c r="H32" s="132" t="s">
         <v>252</v>
       </c>
-      <c r="I32" s="121"/>
-      <c r="J32" s="121"/>
-      <c r="K32" s="121"/>
-      <c r="L32" s="121"/>
-      <c r="M32" s="121"/>
-      <c r="N32" s="121"/>
-      <c r="O32" s="121"/>
-      <c r="P32" s="121"/>
-      <c r="Q32" s="122"/>
+      <c r="I32" s="133"/>
+      <c r="J32" s="133"/>
+      <c r="K32" s="133"/>
+      <c r="L32" s="133"/>
+      <c r="M32" s="133"/>
+      <c r="N32" s="133"/>
+      <c r="O32" s="133"/>
+      <c r="P32" s="133"/>
+      <c r="Q32" s="134"/>
       <c r="R32" s="1"/>
       <c r="S32" s="28" t="e">
         <f>IF(AND($F$24&lt;200,$F$24&gt;=70),"&lt;","")</f>
@@ -37801,27 +37800,27 @@
       <c r="Q34" s="27"/>
     </row>
     <row r="35" spans="2:20" ht="36.75" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="B35" s="117" t="s">
+      <c r="B35" s="129" t="s">
         <v>253</v>
       </c>
-      <c r="C35" s="118"/>
-      <c r="D35" s="119"/>
+      <c r="C35" s="130"/>
+      <c r="D35" s="131"/>
       <c r="F35" s="28" t="e">
         <f>IF($F$24&lt;20,"&gt;","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H35" s="120" t="s">
+      <c r="H35" s="132" t="s">
         <v>254</v>
       </c>
-      <c r="I35" s="121"/>
-      <c r="J35" s="121"/>
-      <c r="K35" s="121"/>
-      <c r="L35" s="121"/>
-      <c r="M35" s="121"/>
-      <c r="N35" s="121"/>
-      <c r="O35" s="121"/>
-      <c r="P35" s="121"/>
-      <c r="Q35" s="122"/>
+      <c r="I35" s="133"/>
+      <c r="J35" s="133"/>
+      <c r="K35" s="133"/>
+      <c r="L35" s="133"/>
+      <c r="M35" s="133"/>
+      <c r="N35" s="133"/>
+      <c r="O35" s="133"/>
+      <c r="P35" s="133"/>
+      <c r="Q35" s="134"/>
       <c r="R35" s="1"/>
       <c r="S35" s="28" t="e">
         <f>IF($F$24&lt;20,"&lt;","")</f>
@@ -37831,22 +37830,22 @@
     </row>
     <row r="36" spans="2:20" ht="5.15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="2:20" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="123"/>
-      <c r="C37" s="123"/>
-      <c r="D37" s="123"/>
-      <c r="E37" s="123"/>
-      <c r="F37" s="123"/>
-      <c r="G37" s="123"/>
-      <c r="H37" s="123"/>
-      <c r="I37" s="123"/>
-      <c r="J37" s="123"/>
-      <c r="K37" s="123"/>
-      <c r="L37" s="123"/>
-      <c r="M37" s="123"/>
-      <c r="N37" s="123"/>
-      <c r="O37" s="123"/>
-      <c r="P37" s="123"/>
-      <c r="Q37" s="123"/>
+      <c r="B37" s="122"/>
+      <c r="C37" s="122"/>
+      <c r="D37" s="122"/>
+      <c r="E37" s="122"/>
+      <c r="F37" s="122"/>
+      <c r="G37" s="122"/>
+      <c r="H37" s="122"/>
+      <c r="I37" s="122"/>
+      <c r="J37" s="122"/>
+      <c r="K37" s="122"/>
+      <c r="L37" s="122"/>
+      <c r="M37" s="122"/>
+      <c r="N37" s="122"/>
+      <c r="O37" s="122"/>
+      <c r="P37" s="122"/>
+      <c r="Q37" s="122"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
@@ -37866,12 +37865,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:T2"/>
-    <mergeCell ref="B3:Q3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="H24:Q24"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="H35:Q35"/>
     <mergeCell ref="B37:Q37"/>
@@ -37883,6 +37876,12 @@
     <mergeCell ref="H32:Q32"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="H28:Q28"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:T2"/>
+    <mergeCell ref="B3:Q3"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="H24:Q24"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.9055118110236221" right="0.74803149606299213" top="0.74803149606299213" bottom="0.6692913385826772" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -39286,20 +39285,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ee15a44e-0948-420d-96df-d16ce70ffded" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ee15a44e-0948-420d-96df-d16ce70ffded" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -39322,6 +39321,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EE14A1C-5FB1-4FE4-BBAD-C2D265A18624}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FD52C5A-C1F0-4A58-ABE1-434C0069F4B0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="ee15a44e-0948-420d-96df-d16ce70ffded"/>
@@ -39336,12 +39343,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EE14A1C-5FB1-4FE4-BBAD-C2D265A18624}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>